<commit_message>
feat: implement explorer breadcrumb trail and enhance navigation in viewer
This commit introduces a new breadcrumb trail feature for the explorer navigation, allowing users to see a full ancestor trail, including implementation references. It adds the `explorerCrumbPath` and `explorerCrumbFromFound` functions to manage breadcrumb generation, improving user experience by providing clearer navigation context. The JavaScript functions are updated to utilize this breadcrumb trail in various sections, ensuring consistency across the viewer. Additionally, tests are added to verify the correct implementation of the breadcrumb functionality, enhancing overall navigation clarity.
</commit_message>
<xml_diff>
--- a/tmp/requirements.xlsx
+++ b/tmp/requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bons1\IdeaProjects\moex-data-model\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB7C1A8-0E50-4D53-B13D-B80740D18FFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D941B7B-7E49-4890-ACD4-A6EB931DBD5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-612" yWindow="1356" windowWidth="41196" windowHeight="16152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="408" windowWidth="41196" windowHeight="16152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="requirements" sheetId="1" r:id="rId1"/>
@@ -712,9 +712,6 @@
     <t>title/name/description/lifecycle и ownership.</t>
   </si>
   <si>
-    <t>У логической сущности должны быть русское бизнес-название, техническое имя, разрешимое эталонное определение (own description либо наследование по ADR-025), статус жизненного цикла и ответственный за данные либо наследование ответственности (ADR-023).</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
@@ -817,9 +814,6 @@
     <t>Status-driven conceptual alignment.</t>
   </si>
   <si>
-    <t>Логическая сущность должна быть прослеживаемо связана с корпоративным понятием либо иметь допустимый статус выравнивания с обоснованием: «ожидает решения», «только локальный смысл» или «не применимо» (только для технических сущностей). Ссылка на корпоративное понятие и пояснение характера реализации могут присутствовать одновременно.</t>
-  </si>
-  <si>
     <t>LDM-006.c1</t>
   </si>
   <si>
@@ -1067,6 +1061,12 @@
   </si>
   <si>
     <t>Пакет не должен иметь посторонних включений, не описанных в спецификации модели решения</t>
+  </si>
+  <si>
+    <t>У логической сущности должны быть русское бизнес-название, техническое имя, разрешимое эталонное определение, статус жизненного цикла и ответственный за данные.</t>
+  </si>
+  <si>
+    <t>Логическая сущность должна быть прослеживаемо связана с сущностью концептуальной модели либо иметь допустимый статус выравнивания с обоснованием: «ожидает решения» или «не применимо».</t>
   </si>
 </sst>
 </file>
@@ -1577,7 +1577,7 @@
         <v>29</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>30</v>
@@ -2041,7 +2041,7 @@
         <v>112</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>113</v>
@@ -2527,7 +2527,7 @@
         <v>190</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>113</v>
@@ -2587,7 +2587,7 @@
         <v>199</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>113</v>
@@ -2774,8 +2774,8 @@
       <c r="H22" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="I22" s="3" t="s">
-        <v>229</v>
+      <c r="I22" s="5" t="s">
+        <v>346</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>113</v>
@@ -2794,19 +2794,19 @@
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
       <c r="R22" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="S22" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="S22" s="3" t="s">
+      <c r="T22" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="T22" s="3" t="s">
+      <c r="U22" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="U22" s="2" t="s">
+      <c r="V22" s="3" t="s">
         <v>233</v>
-      </c>
-      <c r="V22" s="3" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="23" spans="1:22" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -2820,22 +2820,22 @@
         <v>107</v>
       </c>
       <c r="D23" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="G23" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="H23" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="I23" s="4" t="s">
         <v>239</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>240</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>113</v>
@@ -2857,7 +2857,7 @@
         <v>33</v>
       </c>
       <c r="S23" s="3" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="T23" s="3" t="s">
         <v>35</v>
@@ -2866,7 +2866,7 @@
         <v>36</v>
       </c>
       <c r="V23" s="3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="24" spans="1:22" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -2880,22 +2880,22 @@
         <v>107</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="G24" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="H24" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="I24" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>248</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>113</v>
@@ -2917,7 +2917,7 @@
         <v>44</v>
       </c>
       <c r="S24" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="T24" s="3" t="s">
         <v>125</v>
@@ -2926,7 +2926,7 @@
         <v>76</v>
       </c>
       <c r="V24" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="25" spans="1:22" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -2940,22 +2940,22 @@
         <v>107</v>
       </c>
       <c r="D25" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="G25" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="G25" s="3" t="s">
+      <c r="H25" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="I25" s="5" t="s">
         <v>255</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>256</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>113</v>
@@ -2977,7 +2977,7 @@
         <v>44</v>
       </c>
       <c r="S25" s="3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="T25" s="3" t="s">
         <v>125</v>
@@ -2986,7 +2986,7 @@
         <v>76</v>
       </c>
       <c r="V25" s="3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -3000,22 +3000,22 @@
         <v>107</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="G26" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="H26" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="H26" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>264</v>
+      <c r="I26" s="5" t="s">
+        <v>347</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>113</v>
@@ -3037,7 +3037,7 @@
         <v>44</v>
       </c>
       <c r="S26" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="T26" s="3" t="s">
         <v>125</v>
@@ -3046,7 +3046,7 @@
         <v>76</v>
       </c>
       <c r="V26" s="3" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -3060,22 +3060,22 @@
         <v>107</v>
       </c>
       <c r="D27" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="G27" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="H27" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="I27" s="4" t="s">
         <v>270</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="I27" s="3" t="s">
-        <v>272</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>113</v>
@@ -3097,7 +3097,7 @@
         <v>44</v>
       </c>
       <c r="S27" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="T27" s="3" t="s">
         <v>125</v>
@@ -3106,7 +3106,7 @@
         <v>76</v>
       </c>
       <c r="V27" s="3" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -3120,22 +3120,22 @@
         <v>107</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="G28" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="H28" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="I28" s="3" t="s">
         <v>278</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>280</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>113</v>
@@ -3157,7 +3157,7 @@
         <v>44</v>
       </c>
       <c r="S28" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="T28" s="3" t="s">
         <v>125</v>
@@ -3166,7 +3166,7 @@
         <v>47</v>
       </c>
       <c r="V28" s="3" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="29" spans="1:22" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -3180,22 +3180,22 @@
         <v>107</v>
       </c>
       <c r="D29" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="G29" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="H29" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="I29" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>288</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>113</v>
@@ -3217,7 +3217,7 @@
         <v>63</v>
       </c>
       <c r="S29" s="3" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="T29" s="3" t="s">
         <v>65</v>
@@ -3226,7 +3226,7 @@
         <v>66</v>
       </c>
       <c r="V29" s="3" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="30" spans="1:22" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -3240,22 +3240,22 @@
         <v>107</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="G30" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="H30" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="G30" s="3" t="s">
+      <c r="I30" s="3" t="s">
         <v>294</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>296</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>113</v>
@@ -3267,7 +3267,7 @@
         <v>32</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -3277,7 +3277,7 @@
         <v>33</v>
       </c>
       <c r="S30" s="3" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="T30" s="3" t="s">
         <v>35</v>
@@ -3286,7 +3286,7 @@
         <v>36</v>
       </c>
       <c r="V30" s="3" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="31" spans="1:22" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -3300,22 +3300,22 @@
         <v>107</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="G31" s="3" t="s">
         <v>301</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="H31" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="I31" s="3" t="s">
         <v>303</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>305</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>113</v>
@@ -3339,7 +3339,7 @@
         <v>44</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="T31" s="3" t="s">
         <v>125</v>
@@ -3348,7 +3348,7 @@
         <v>76</v>
       </c>
       <c r="V31" s="3" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="32" spans="1:22" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -3362,22 +3362,22 @@
         <v>107</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="G32" s="3" t="s">
         <v>309</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="H32" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="I32" s="3" t="s">
         <v>311</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="I32" s="3" t="s">
-        <v>313</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>113</v>
@@ -3389,7 +3389,7 @@
         <v>32</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -3399,7 +3399,7 @@
         <v>44</v>
       </c>
       <c r="S32" s="3" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="T32" s="3" t="s">
         <v>125</v>
@@ -3408,7 +3408,7 @@
         <v>76</v>
       </c>
       <c r="V32" s="3" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="33" spans="1:22" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -3422,22 +3422,22 @@
         <v>107</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="G33" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="H33" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="I33" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="I33" s="3" t="s">
-        <v>321</v>
       </c>
       <c r="J33" s="2" t="s">
         <v>113</v>
@@ -3449,7 +3449,7 @@
         <v>32</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -3459,7 +3459,7 @@
         <v>33</v>
       </c>
       <c r="S33" s="3" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="T33" s="3" t="s">
         <v>95</v>
@@ -3468,7 +3468,7 @@
         <v>36</v>
       </c>
       <c r="V33" s="3" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="34" spans="1:22" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -3482,22 +3482,22 @@
         <v>107</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="G34" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="H34" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="I34" s="3" t="s">
         <v>328</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>330</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>113</v>
@@ -3509,7 +3509,7 @@
         <v>32</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -3519,7 +3519,7 @@
         <v>44</v>
       </c>
       <c r="S34" s="3" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="T34" s="3" t="s">
         <v>125</v>
@@ -3528,7 +3528,7 @@
         <v>76</v>
       </c>
       <c r="V34" s="3" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="35" spans="1:22" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -3542,22 +3542,22 @@
         <v>107</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="G35" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="H35" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="G35" s="3" t="s">
+      <c r="I35" s="3" t="s">
         <v>336</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="I35" s="3" t="s">
-        <v>338</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>113</v>
@@ -3569,7 +3569,7 @@
         <v>32</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -3579,7 +3579,7 @@
         <v>44</v>
       </c>
       <c r="S35" s="3" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="T35" s="3" t="s">
         <v>125</v>
@@ -3588,23 +3588,23 @@
         <v>47</v>
       </c>
       <c r="V35" s="3" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="36" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
       <c r="E36" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="37" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="E37" s="2" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>113</v>

</xml_diff>